<commit_message>
Remove MIN_STOP_PCT e MIN_RR_RATIO forcing em pivot levels
A pedido do usuario, respeita exatamente os levels de pivot/s1/r1 sem
forcar stop minimo (2%) ou extensao de alvo por R:R minimo (1.5).

Mudancas em ga_run.py (apply phase pivot section):
- Stop: s1 * 0.995 diretamente (sem floor MIN_STOP_PCT)
  Fallback ATR so se s1 >= best_buy (caso raro)
  Ultimo fallback 1% se tudo falhar (evita stop invalido)
- Alvo: r1 * 0.998 diretamente (sem forcar extensao se rr < 1.5)
  Se r1 <= best_buy, mantem take_profit ATR-based anterior
- R:R calculado informativamente (rr_display), nao usado para ajuste

Resultado verificado em summary_latest.xlsx:
  CMIG4: rr=0.8 (antes forcado para 1.5)
  MULT3: stop=1.86% (antes forcado para 2%)
  MULT3: rr=2.1 (aumentou porque stop apertou sem floor)
  HGBS11: stop=2.00% (s1 realmente a essa distancia)
  Todos os niveis agora refletem pivot/s1/r1 originais.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/summary_latest_v2.xlsx
+++ b/summary_latest_v2.xlsx
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>AGUARDAR ROMPER PIVOT @33.81 * S2 Alta momentum * +3.9% alvo @34.36 (WR 75% / alvo 73%) * Stop @32.42 (-2.0%) * Cancelar se &lt; MA50/S1 @32.28</t>
+          <t>AGUARDAR ROMPER PIVOT @33.81 * S2 Alta momentum * +3.9% alvo @34.36 (WR 75% / alvo 73%) * Stop @32.47 (-1.9%) * Cancelar se &lt; MA50/S1 @32.28</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1724,7 +1724,7 @@
         <v>33.915</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>32.4221</v>
+        <v>32.4668</v>
       </c>
       <c r="K13" s="8" t="n">
         <v>34.3611</v>
@@ -1733,7 +1733,7 @@
         <v>32.2805</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>33.81</v>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ORDEM LIMITE @13.11 * S2 Alta momentum * +3.0% alvo @13.50 (WR 67% / alvo 66%) * Stop @12.84 (-2.0%) * Cancelar se &lt; MA50/S1 @11.81</t>
+          <t>ORDEM LIMITE @13.11 * S2 Alta momentum * +2.2% alvo @13.40 (WR 67% / alvo 66%) * Stop @12.75 (-2.7%) * Cancelar se &lt; MA50/S1 @11.81</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>+3.0%</t>
+          <t>+2.2%</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1808,19 +1808,19 @@
         <v>13.1059</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>13.364</v>
+        <v>13.2626</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>12.8438</v>
+        <v>12.7491</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>13.499</v>
+        <v>13.3966</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>11.8072</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>13.2767</v>
@@ -75682,7 +75682,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AGUARDAR ROMPER PIVOT @33.81 * S2 Alta momentum * +3.9% alvo @34.36 (WR 75% / alvo 73%) * Stop @32.42 (-2.0%) * Cancelar se &lt; MA50/S1 @32.28</t>
+          <t>AGUARDAR ROMPER PIVOT @33.81 * S2 Alta momentum * +3.9% alvo @34.36 (WR 75% / alvo 73%) * Stop @32.47 (-1.9%) * Cancelar se &lt; MA50/S1 @32.28</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -75710,7 +75710,7 @@
         <v>33.915</v>
       </c>
       <c r="J13" t="n">
-        <v>32.4221</v>
+        <v>32.4668</v>
       </c>
       <c r="K13" t="n">
         <v>34.3611</v>
@@ -75719,7 +75719,7 @@
         <v>32.2805</v>
       </c>
       <c r="M13" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="N13" t="n">
         <v>33.81</v>
@@ -75787,12 +75787,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ORDEM LIMITE @13.11 * S2 Alta momentum * +3.0% alvo @13.50 (WR 67% / alvo 66%) * Stop @12.84 (-2.0%) * Cancelar se &lt; MA50/S1 @11.81</t>
+          <t>ORDEM LIMITE @13.11 * S2 Alta momentum * +2.2% alvo @13.40 (WR 67% / alvo 66%) * Stop @12.75 (-2.7%) * Cancelar se &lt; MA50/S1 @11.81</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+3.0%</t>
+          <t>+2.2%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -75812,19 +75812,19 @@
         <v>13.1059</v>
       </c>
       <c r="I14" t="n">
-        <v>13.364</v>
+        <v>13.2626</v>
       </c>
       <c r="J14" t="n">
-        <v>12.8438</v>
+        <v>12.7491</v>
       </c>
       <c r="K14" t="n">
-        <v>13.499</v>
+        <v>13.3966</v>
       </c>
       <c r="L14" t="n">
         <v>11.8072</v>
       </c>
       <c r="M14" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="N14" t="n">
         <v>13.2767</v>

</xml_diff>